<commit_message>
Error in table 1 fixed
</commit_message>
<xml_diff>
--- a/Agg_tables/table1_comparison.xlsx
+++ b/Agg_tables/table1_comparison.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Tiedostot\Vaikkari\Export\Root_Export_20260204\Tulokset_HUS442021_TietoAllasTutkimusToisio_HUS-1915-2021-Rintasyopahoitojen-vaikuttavuus_04022026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Tiedostot\Vaikkari\Git_repo\Transportability-of-Neoadjuvant-HER2-Positive-Breast-Cancer-Trial-Outcomes\Agg_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301A92E0-10E3-4C03-B82F-0DCC287A74ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FE03DD-8155-45FE-96F0-E78F3B5CE4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{93AFF125-A546-48B0-988B-26716797AFB4}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="9960" xr2:uid="{93AFF125-A546-48B0-988B-26716797AFB4}"/>
   </bookViews>
   <sheets>
     <sheet name="table1" sheetId="2" r:id="rId1"/>
@@ -324,9 +324,6 @@
     <t>79 % [73 % - 84 %]</t>
   </si>
   <si>
-    <t>16 % [3 % - 8 %]</t>
-  </si>
-  <si>
     <t>22 % [17 % - 27 %]</t>
   </si>
   <si>
@@ -430,6 +427,9 @@
   </si>
   <si>
     <t>2 % [0 % - 4 %]</t>
+  </si>
+  <si>
+    <t>16 % [12 % - 21 %]</t>
   </si>
 </sst>
 </file>
@@ -465,13 +465,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -836,23 +835,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE927D1B-1C2A-49A2-B28C-ED08FE2B0F0A}">
   <dimension ref="A1:L69"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="52" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -881,16 +880,16 @@
         <v>55</v>
       </c>
       <c r="J1" t="s">
+        <v>101</v>
+      </c>
+      <c r="K1" t="s">
         <v>102</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>103</v>
       </c>
-      <c r="L1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -926,10 +925,10 @@
         <v>221</v>
       </c>
       <c r="L2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -949,10 +948,10 @@
         <v>40</v>
       </c>
       <c r="K3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -969,7 +968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>61</v>
       </c>
@@ -977,7 +976,7 @@
         <v>58</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D5" t="str">
         <f>table1[[#This Row],[HUS Variable]]</f>
@@ -1000,7 +999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>62</v>
       </c>
@@ -1008,11 +1007,11 @@
         <v>143</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>63</v>
       </c>
@@ -1020,11 +1019,11 @@
         <v>19</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F8" s="1"/>
       <c r="G8" t="s">
         <v>59</v>
@@ -1036,7 +1035,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F9" s="1"/>
       <c r="G9" t="s">
         <v>60</v>
@@ -1048,7 +1047,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1078,7 +1077,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1109,16 +1108,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
       <c r="B12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" t="s">
         <v>117</v>
       </c>
-      <c r="C12" t="s">
-        <v>118</v>
-      </c>
       <c r="D12" t="str">
         <f>table1[[#This Row],[HUS Variable]]</f>
         <v>ECOG: 2</v>
@@ -1140,7 +1139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1171,7 +1170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -1201,7 +1200,7 @@
         <v>0.73</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -1231,7 +1230,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1252,7 +1251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
         <v>44</v>
       </c>
@@ -1263,7 +1262,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
         <v>45</v>
       </c>
@@ -1274,7 +1273,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
         <v>46</v>
       </c>
@@ -1285,10 +1284,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F20" s="1"/>
       <c r="J20" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -1297,10 +1296,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F21" s="1"/>
       <c r="J21" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K21">
         <v>221</v>
@@ -1309,7 +1308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1350,7 +1349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -1391,7 +1390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -1432,7 +1431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1443,7 +1442,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -1454,7 +1453,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>14</v>
       </c>
@@ -1465,12 +1464,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C28" t="s">
         <v>73</v>
@@ -1486,7 +1485,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -1507,7 +1506,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -1528,7 +1527,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -1549,7 +1548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>64</v>
       </c>
@@ -1570,7 +1569,7 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1591,7 +1590,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>66</v>
       </c>
@@ -1599,7 +1598,7 @@
         <v>44</v>
       </c>
       <c r="C34" t="s">
-        <v>92</v>
+        <v>127</v>
       </c>
       <c r="G34" t="str">
         <f>table1[[#This Row],[HUS Variable]]</f>
@@ -1612,7 +1611,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -1653,7 +1652,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -1694,7 +1693,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -1735,7 +1734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>22</v>
       </c>
@@ -1746,7 +1745,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -1757,7 +1756,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>24</v>
       </c>
@@ -1765,19 +1764,19 @@
         <v>21</v>
       </c>
       <c r="C40" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>25</v>
       </c>
       <c r="B41" t="s">
+        <v>116</v>
+      </c>
+      <c r="C41" t="s">
         <v>117</v>
       </c>
-      <c r="C41" t="s">
-        <v>118</v>
-      </c>
       <c r="J41" t="str">
         <f>table1[[#This Row],[HUS Variable]]</f>
         <v>IHC: 1+</v>
@@ -1789,7 +1788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -1800,7 +1799,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>27</v>
       </c>
@@ -1811,7 +1810,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -1832,14 +1831,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>119</v>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>118</v>
       </c>
       <c r="B45">
         <v>183</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" t="s">
         <v>85</v>
       </c>
       <c r="G45" t="str">
@@ -1854,18 +1853,18 @@
       </c>
       <c r="L45" s="1"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>120</v>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>119</v>
       </c>
       <c r="B46">
         <v>71</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" t="s">
         <v>77</v>
       </c>
       <c r="G46" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H46">
         <v>104</v>
@@ -1875,15 +1874,15 @@
       </c>
       <c r="L46" s="1"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>121</v>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>120</v>
       </c>
       <c r="B47">
         <v>14</v>
       </c>
-      <c r="C47" s="3" t="s">
-        <v>123</v>
+      <c r="C47" t="s">
+        <v>122</v>
       </c>
       <c r="G47" t="str">
         <f>table1[[#This Row],[HUS Variable]]</f>
@@ -1897,9 +1896,9 @@
       </c>
       <c r="L47" s="1"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>122</v>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>121</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -1919,7 +1918,7 @@
       </c>
       <c r="L48" s="1"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>29</v>
       </c>
@@ -1930,7 +1929,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -1941,7 +1940,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" t="str">
         <f>table1[[#This Row],[HELEN-006 Variable]]</f>
         <v>Ki-67 index &lt;= 30 %</v>
@@ -1950,10 +1949,10 @@
         <v>172</v>
       </c>
       <c r="C51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G51" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H51">
         <v>75</v>
@@ -1962,7 +1961,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" t="str">
         <f>table1[[#This Row],[HELEN-006 Variable]]</f>
         <v>Ki-67 index &gt; 30 %</v>
@@ -1971,10 +1970,10 @@
         <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G52" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H52">
         <v>262</v>
@@ -1983,21 +1982,21 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
-        <v>124</v>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>123</v>
       </c>
       <c r="B53">
         <v>5</v>
       </c>
-      <c r="C53" s="3" t="s">
-        <v>127</v>
+      <c r="C53" t="s">
+        <v>126</v>
       </c>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D54" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E54">
         <v>65</v>
@@ -2006,9 +2005,9 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D55" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E55">
         <v>32</v>
@@ -2017,9 +2016,9 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D56" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E56">
         <v>10</v>
@@ -2028,10 +2027,10 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F57" s="1"/>
       <c r="G57" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H57">
         <v>212</v>
@@ -2040,10 +2039,10 @@
         <v>0.63</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F58" s="1"/>
       <c r="G58" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H58">
         <v>125</v>
@@ -2052,11 +2051,11 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F59" s="1"/>
       <c r="I59" s="1"/>
       <c r="J59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K59">
         <v>183</v>
@@ -2065,11 +2064,11 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F60" s="1"/>
       <c r="I60" s="1"/>
       <c r="J60" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K60">
         <v>38</v>
@@ -2078,7 +2077,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D61" t="s">
         <v>47</v>
       </c>
@@ -2109,7 +2108,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D62" t="s">
         <v>48</v>
       </c>
@@ -2140,7 +2139,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D63" t="s">
         <v>49</v>
       </c>
@@ -2171,7 +2170,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D64" t="s">
         <v>50</v>
       </c>
@@ -2202,11 +2201,11 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="65" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F65" s="1"/>
       <c r="I65" s="1"/>
       <c r="J65" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K65">
         <v>54</v>
@@ -2215,11 +2214,11 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="66" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F66" s="1"/>
       <c r="I66" s="1"/>
       <c r="J66" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K66">
         <v>84</v>
@@ -2228,11 +2227,11 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="67" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F67" s="1"/>
       <c r="I67" s="1"/>
       <c r="J67" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K67">
         <v>83</v>
@@ -2241,7 +2240,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="68" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="6:12" x14ac:dyDescent="0.3">
       <c r="G68" t="s">
         <v>57</v>
       </c>
@@ -2252,7 +2251,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="69" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="6:12" x14ac:dyDescent="0.3">
       <c r="G69" t="s">
         <v>58</v>
       </c>
@@ -2274,7 +2273,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF7CAB12-00B3-49CA-92AA-9D4B7E9ADE85}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>